<commit_message>
finish py and update jupyter notebook
</commit_message>
<xml_diff>
--- a/hwk4/test_data.xlsx
+++ b/hwk4/test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yushuo Ruan\Dropbox\Spring2019\RecommenderSystems\Gitrepo\hwk4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2ED80F-AAD7-434B-A0B0-CBB1835CE44A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD85F8D9-03AD-45CD-910B-07DA45CF102C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10935" yWindow="2445" windowWidth="21180" windowHeight="16425" firstSheet="2" activeTab="4" xr2:uid="{D8D605F8-015C-0740-BF92-A813C61E88C3}"/>
+    <workbookView xWindow="10935" yWindow="2445" windowWidth="21180" windowHeight="16425" firstSheet="2" activeTab="5" xr2:uid="{D8D605F8-015C-0740-BF92-A813C61E88C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Rating Data" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="35">
   <si>
     <t>User</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>P(~f|L)</t>
+  </si>
+  <si>
+    <t>like</t>
   </si>
 </sst>
 </file>
@@ -151,7 +154,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -174,12 +177,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF7E00"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -228,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -239,7 +236,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1306,7 +1302,8 @@
       <c r="F2">
         <v>2</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="8">
+        <f>(2+0.01)/(4+0.02)</f>
         <v>0.5</v>
       </c>
       <c r="H2" t="s">
@@ -1323,8 +1320,9 @@
       <c r="F3">
         <v>1</v>
       </c>
-      <c r="G3" s="6">
-        <v>0.33400000000000002</v>
+      <c r="G3" s="8">
+        <f>(1+0.01)/(3+0.02)</f>
+        <v>0.33443708609271522</v>
       </c>
       <c r="H3" t="s">
         <v>26</v>
@@ -1340,8 +1338,9 @@
       <c r="F4">
         <v>3</v>
       </c>
-      <c r="G4" s="10">
-        <v>0.99668874172184996</v>
+      <c r="G4" s="8">
+        <f>(3+0.01)/(3+0.02)</f>
+        <v>0.99668874172185418</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1359,7 +1358,8 @@
       <c r="F7">
         <v>2</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="8">
+        <f>(2+0.01)/(4+0.02)</f>
         <v>0.5</v>
       </c>
     </row>
@@ -1370,8 +1370,9 @@
       <c r="F8">
         <v>2</v>
       </c>
-      <c r="G8" s="6">
-        <v>0.66666666666666663</v>
+      <c r="G8" s="8">
+        <f>(2+0.01)/(3+0.02)</f>
+        <v>0.66556291390728473</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1381,8 +1382,9 @@
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" s="6">
-        <v>0</v>
+      <c r="G9" s="8">
+        <f>(0+0.01)/(3+0.02)</f>
+        <v>3.3112582781456954E-3</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1643,25 +1645,91 @@
       <c r="B19" t="s">
         <v>32</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="8">
         <f>(C12+0.02)/(2+0.04)</f>
         <v>0.5</v>
       </c>
-      <c r="G19" s="9"/>
+      <c r="D19" s="8">
+        <f t="shared" ref="D19:L19" si="0">(D12+0.02)/(2+0.04)</f>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="E19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="G19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="H19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="I19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="J19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="K19" s="8">
+        <f t="shared" si="0"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="L19" s="8">
+        <f t="shared" si="0"/>
+        <v>0.99019607843137258</v>
+      </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
+      <c r="C20" s="8">
+        <f>(C13+0.02)/(2+0.04)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D20" s="8">
+        <f t="shared" ref="D20:L21" si="1">(D13+0.02)/(2+0.04)</f>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="E20" s="8">
+        <f t="shared" si="1"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="F20" s="8">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="G20" s="8">
+        <f t="shared" si="1"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="H20" s="8">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="I20" s="8">
+        <f t="shared" si="1"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="J20" s="8">
+        <f t="shared" si="1"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="K20" s="8">
+        <f t="shared" si="1"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="L20" s="8">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1670,13 +1738,91 @@
       <c r="B21" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="9"/>
+      <c r="C21" s="8">
+        <f>(C14+0.02)/(1+0.04)</f>
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="D21" s="8">
+        <f t="shared" ref="D21:L21" si="2">(D14+0.02)/(1+0.04)</f>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="2"/>
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="F21" s="8">
+        <f t="shared" si="2"/>
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="G21" s="8">
+        <f t="shared" si="2"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="H21" s="8">
+        <f t="shared" si="2"/>
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="I21" s="8">
+        <f t="shared" si="2"/>
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="J21" s="8">
+        <f t="shared" si="2"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="K21" s="8">
+        <f t="shared" si="2"/>
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="L21" s="8">
+        <f t="shared" si="2"/>
+        <v>0.98076923076923073</v>
+      </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>33</v>
       </c>
-      <c r="G22" s="9"/>
+      <c r="C22" s="8">
+        <f>(C15+0.02)/(2+0.04)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="8">
+        <f t="shared" ref="D22:L22" si="3">(D15+0.02)/(2+0.04)</f>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="E22" s="8">
+        <f t="shared" si="3"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="F22" s="8">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="G22" s="8">
+        <f t="shared" si="3"/>
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="H22" s="8">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="I22" s="8">
+        <f t="shared" si="3"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="J22" s="8">
+        <f t="shared" si="3"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="K22" s="8">
+        <f t="shared" si="3"/>
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="L22" s="8">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1685,29 +1831,91 @@
       <c r="B23" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
+      <c r="C23" s="8">
+        <f>(C16+0.02)/(3+0.04)</f>
+        <v>0.99342105263157898</v>
+      </c>
+      <c r="D23" s="8">
+        <f t="shared" ref="D23:L23" si="4">(D16+0.02)/(3+0.04)</f>
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="E23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="F23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="G23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.33552631578947367</v>
+      </c>
+      <c r="H23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="I23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="J23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.33552631578947367</v>
+      </c>
+      <c r="K23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.33552631578947367</v>
+      </c>
+      <c r="L23" s="8">
+        <f t="shared" si="4"/>
+        <v>0.66447368421052633</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
+      <c r="C24" s="8">
+        <f>(C17+0.02)/(0+0.04)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="8">
+        <f t="shared" ref="D24:L24" si="5">(D17+0.02)/(0+0.04)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="F24" s="8">
+        <f>(F17+0.02)/(0+0.04)</f>
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="I24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="J24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="K24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="L24" s="8">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1717,7 +1925,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D6F5FD9-3BB6-7B4A-AE4C-B18D86A2FD18}">
-  <dimension ref="A3:H24"/>
+  <dimension ref="A3:H25"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.125" customWidth="1"/>
@@ -1763,26 +1971,80 @@
       <c r="A5" t="s">
         <v>28</v>
       </c>
+      <c r="B5" s="8">
+        <f>(1+0.01)/(3+0.02)</f>
+        <v>0.33443708609271522</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.98076923076923073</v>
+      </c>
+      <c r="G5" s="8">
+        <v>1.9230769230769232E-2</v>
+      </c>
+      <c r="H5" s="8">
+        <v>1.9230769230769232E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
+      <c r="B6" s="8">
+        <f>(2+0.01)/(3+0.02)</f>
+        <v>0.66556291390728473</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="8">
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="E6" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="G6" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="H6" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
+      <c r="B7" s="7">
+        <f>PRODUCT(B5:H5)/PRODUCT(B6:H6)</f>
+        <v>14.452902983343396</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="8"/>
+      <c r="B8" s="8">
+        <f>LN(B7)</f>
+        <v>2.6708952928823129</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1823,28 +2085,81 @@
       <c r="A13" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="6"/>
+      <c r="B13" s="8">
+        <f>(2+0.01)/(4+0.02)</f>
+        <v>0.5</v>
+      </c>
+      <c r="C13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="E13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="8">
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="G13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="H13" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="H14" s="6"/>
+      <c r="B14" s="8">
+        <f>(2+0.01)/(4+0.02)</f>
+        <v>0.5</v>
+      </c>
+      <c r="C14" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="8">
+        <v>0.99019607843137258</v>
+      </c>
+      <c r="E14" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="G14" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
+      <c r="H14" s="8">
+        <v>9.8039215686274508E-3</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
+      <c r="B15" s="7">
+        <f>PRODUCT(B13:H13)/PRODUCT(B14:H14)</f>
+        <v>51</v>
+      </c>
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
+      <c r="B16" s="7">
+        <f>LN(B15)</f>
+        <v>3.9318256327243257</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1879,20 +2194,68 @@
       <c r="A21" t="s">
         <v>28</v>
       </c>
+      <c r="B21" s="8">
+        <f>(3+0.01)/(3+0.02)</f>
+        <v>0.99668874172185418</v>
+      </c>
+      <c r="C21" s="8">
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0.66447368421052633</v>
+      </c>
+      <c r="E21" s="8">
+        <v>0.33552631578947367</v>
+      </c>
+      <c r="F21" s="8">
+        <v>0.66447368421052633</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>29</v>
       </c>
+      <c r="B22" s="8">
+        <f>(0+0.01)/(3+0.02)</f>
+        <v>3.3112582781456954E-3</v>
+      </c>
+      <c r="C22" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="E22" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="B23" s="7">
+        <f>PRODUCT(B21:H21)/PRODUCT(B22:H22)</f>
+        <v>474.07431250887225</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>3</v>
+        <v>27</v>
+      </c>
+      <c r="B24" s="7">
+        <f>LN(B23)</f>
+        <v>6.1613640868516555</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>